<commit_message>
chore: snapshot before repository cleanup
</commit_message>
<xml_diff>
--- a/Info_extractor/data_extraction_template_v2.xlsx
+++ b/Info_extractor/data_extraction_template_v2.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -520,132 +520,137 @@
           <t>Is_Multicenter</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Centers</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Countries</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Enrollment_Start</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Enrollment_End</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Registry_ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Intervention_Type</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Comparator</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>N_Intervention</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>N_Control</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>N_Total</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Donor_Type</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>ECD_Definition</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>ECD_Percentage</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Donor_Age_Int</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Donor_Age_Ctrl</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Donor_BMI_Int</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Donor_BMI_Ctrl</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>DRI_Type</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>DRI_Int</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>DRI_Ctrl</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Recipient_Age_Int</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Recipient_Age_Ctrl</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>MELD_Int</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>MELD_Ctrl</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Matching_Method</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Matching_Variables</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -914,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EC1"/>
+  <dimension ref="A1:GK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1696,6 +1701,306 @@
           <t>PRS_Source_Location</t>
         </is>
       </c>
+      <c r="ED1" t="inlineStr">
+        <is>
+          <t>GS_30d_Reported</t>
+        </is>
+      </c>
+      <c r="EE1" t="inlineStr">
+        <is>
+          <t>GS_30d_Int_Events</t>
+        </is>
+      </c>
+      <c r="EF1" t="inlineStr">
+        <is>
+          <t>GS_30d_Int_Total</t>
+        </is>
+      </c>
+      <c r="EG1" t="inlineStr">
+        <is>
+          <t>GS_30d_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>GS_30d_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>GS_30d_Source</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>GS_90d_Reported</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>GS_90d_Int_Events</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>GS_90d_Int_Total</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>GS_90d_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>GS_90d_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
+          <t>GS_90d_Source</t>
+        </is>
+      </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Reported</t>
+        </is>
+      </c>
+      <c r="EQ1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="ER1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="ES1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="ET1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="EU1" t="inlineStr">
+        <is>
+          <t>GS_1yr_Source</t>
+        </is>
+      </c>
+      <c r="EV1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Reported</t>
+        </is>
+      </c>
+      <c r="EW1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="EX1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="EY1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="EZ1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="FA1" t="inlineStr">
+        <is>
+          <t>GS_3yr_Source</t>
+        </is>
+      </c>
+      <c r="FB1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Reported</t>
+        </is>
+      </c>
+      <c r="FC1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="FD1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="FE1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="FG1" t="inlineStr">
+        <is>
+          <t>GS_5yr_Source</t>
+        </is>
+      </c>
+      <c r="FH1" t="inlineStr">
+        <is>
+          <t>PS_30d_Reported</t>
+        </is>
+      </c>
+      <c r="FI1" t="inlineStr">
+        <is>
+          <t>PS_30d_Int_Events</t>
+        </is>
+      </c>
+      <c r="FJ1" t="inlineStr">
+        <is>
+          <t>PS_30d_Int_Total</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>PS_30d_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>PS_30d_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>PS_30d_Source</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>PS_90d_Reported</t>
+        </is>
+      </c>
+      <c r="FO1" t="inlineStr">
+        <is>
+          <t>PS_90d_Int_Events</t>
+        </is>
+      </c>
+      <c r="FP1" t="inlineStr">
+        <is>
+          <t>PS_90d_Int_Total</t>
+        </is>
+      </c>
+      <c r="FQ1" t="inlineStr">
+        <is>
+          <t>PS_90d_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="FR1" t="inlineStr">
+        <is>
+          <t>PS_90d_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>PS_90d_Source</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Reported</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="FW1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="FX1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="FY1" t="inlineStr">
+        <is>
+          <t>PS_1yr_Source</t>
+        </is>
+      </c>
+      <c r="FZ1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Reported</t>
+        </is>
+      </c>
+      <c r="GA1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="GB1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="GC1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="GD1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="GE1" t="inlineStr">
+        <is>
+          <t>PS_3yr_Source</t>
+        </is>
+      </c>
+      <c r="GF1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Reported</t>
+        </is>
+      </c>
+      <c r="GG1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Int_Events</t>
+        </is>
+      </c>
+      <c r="GH1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Int_Total</t>
+        </is>
+      </c>
+      <c r="GI1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Ctrl_Events</t>
+        </is>
+      </c>
+      <c r="GJ1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Ctrl_Total</t>
+        </is>
+      </c>
+      <c r="GK1" t="inlineStr">
+        <is>
+          <t>PS_5yr_Source</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>